<commit_message>
Fill the alternate mobile in the Selloship file
Selloship rejected every upload with "Row No 2 : Alternate Mobile No is
invalid" because the column went out blank. Creators give one number, so the
same number now serves as the alternate.

Also added a fallback email under Setup, empty by default and used only when a
creator gave none — a blank email is the next most likely rejection, and this
turns it into filling one field rather than a code change.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014hWLHcPsqiVrX7Q6P25P8A
</commit_message>
<xml_diff>
--- a/templates/selloship-bulk-order-sample.xlsx
+++ b/templates/selloship-bulk-order-sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:U3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Aravi Organic Rosemary Lavender Hair Oil - 200 ml + Aravi Organic Sunscreen Body Lotion SPF50 - 200 ml</v>
+        <v>Body wash</v>
       </c>
       <c r="B2">
         <v>500</v>
@@ -475,46 +475,46 @@
         <v>500</v>
       </c>
       <c r="D2" t="str">
-        <v>Mridula</v>
+        <v>Monidipa</v>
       </c>
       <c r="E2" t="str">
-        <v>Sharma</v>
+        <v>.</v>
       </c>
       <c r="F2" t="str">
-        <v>8302605158</v>
+        <v>9239550041</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>9239550041</v>
       </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>621, G-2 krishna residency, road no. 05, Devi nagar sodala</v>
+        <v>House of Chandrasova</v>
       </c>
       <c r="J2" t="str">
-        <v>Rajasthan</v>
+        <v>West Bengal</v>
       </c>
       <c r="K2" t="str">
-        <v>Jaipur</v>
+        <v>Bardhaman</v>
       </c>
       <c r="L2" t="str">
-        <v>302019</v>
+        <v>713103</v>
       </c>
       <c r="M2" t="str">
-        <v>Devi nagar sodala</v>
+        <v>.</v>
       </c>
       <c r="N2">
         <v>4</v>
       </c>
       <c r="O2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="str">
         <v>PR632</v>
       </c>
       <c r="Q2" t="str">
-        <v>AO/HO/RosemaryLavender/200 | AO/SS/BodyLotion</v>
+        <v>AO/BWash/Salicylic/300</v>
       </c>
       <c r="R2" t="str">
         <v/>
@@ -531,7 +531,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Aravi Organic 2% Salicylic Bodywash - 300 ml + Aravi Organic 20% Urea Foot Roll On - 50 ml</v>
+        <v>Body wash</v>
       </c>
       <c r="B3">
         <v>500</v>
@@ -540,31 +540,31 @@
         <v>500</v>
       </c>
       <c r="D3" t="str">
-        <v>Neha</v>
+        <v>Mridula</v>
       </c>
       <c r="E3" t="str">
-        <v>.</v>
+        <v>Sharma</v>
       </c>
       <c r="F3" t="str">
-        <v>8950430375</v>
+        <v>8302605158</v>
       </c>
       <c r="G3" t="str">
-        <v/>
+        <v>8302605158</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>m@example.com</v>
       </c>
       <c r="I3" t="str">
-        <v>noultha didwari road Mohit jeweller</v>
+        <v>621 G-2 Krishna Residency</v>
       </c>
       <c r="J3" t="str">
-        <v>Haryana</v>
+        <v>Rajasthan</v>
       </c>
       <c r="K3" t="str">
-        <v>Panipat</v>
+        <v>Jaipur</v>
       </c>
       <c r="L3" t="str">
-        <v>132145</v>
+        <v>302019</v>
       </c>
       <c r="M3" t="str">
         <v>.</v>
@@ -573,13 +573,13 @@
         <v>4</v>
       </c>
       <c r="O3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P3" t="str">
         <v>PR633</v>
       </c>
       <c r="Q3" t="str">
-        <v>AO/BWash/Salicylic/300 | AO/RO/AB/Foot/50</v>
+        <v>AO/BWash/Salicylic/300</v>
       </c>
       <c r="R3" t="str">
         <v/>
@@ -591,77 +591,12 @@
         <v>20</v>
       </c>
       <c r="U3">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Aravi Organic Rosemary Essential Oil - 15 ml</v>
-      </c>
-      <c r="B4">
-        <v>500</v>
-      </c>
-      <c r="C4">
-        <v>500</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Chhavi</v>
-      </c>
-      <c r="E4" t="str">
-        <v>.</v>
-      </c>
-      <c r="F4" t="str">
-        <v>8951669546</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v>11/119, street no.: 2</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Uttar Pradesh</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Baraut</v>
-      </c>
-      <c r="L4" t="str">
-        <v>250611</v>
-      </c>
-      <c r="M4" t="str">
-        <v>.</v>
-      </c>
-      <c r="N4">
-        <v>4</v>
-      </c>
-      <c r="O4">
-        <v>1</v>
-      </c>
-      <c r="P4" t="str">
-        <v>PR634</v>
-      </c>
-      <c r="Q4" t="str">
-        <v>AO/EO/Rosemary/15</v>
-      </c>
-      <c r="R4" t="str">
-        <v/>
-      </c>
-      <c r="S4">
-        <v>25</v>
-      </c>
-      <c r="T4">
-        <v>20</v>
-      </c>
-      <c r="U4">
         <v>12</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>